<commit_message>
Add Huaxia Publishing House titles to other-publisher list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KLZ8HBrsPXT91pLYmTZE9t
</commit_message>
<xml_diff>
--- a/骨科康复图书_其他出版社汇总.xlsx
+++ b/骨科康复图书_其他出版社汇总.xlsx
@@ -13,7 +13,7 @@
     <sheet name="出版社统计" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">中文出版社!$A$1:$O$64</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">中文出版社!$A$1:$O$69</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">英文出版社!$A$1:$Q$136</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2512" uniqueCount="1386">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2563" uniqueCount="1408">
   <si>
     <t xml:space="preserve">序号</t>
   </si>
@@ -14600,6 +14600,163 @@
     <t xml:space="preserve">华夏出版社</t>
   </si>
   <si>
+    <t xml:space="preserve">骨盆平衡技术</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">齐鸿</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">邓宁 主编</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">978-7-5080-9763-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hxph.com.cn/newBooks/9475.jhtml</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">实用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PNF</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">治疗</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">美</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) Susan S. Adler, (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">比</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) Dominiek Beckers, (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">荷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) Math Buck </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">著</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">刘钦刚</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNF in Practice: An Illustrated Guide (4th ed.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">978-7-5080-9391-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hxph.com.cn/newBooks/8974.jhtml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">临床运动疗法学</t>
+  </si>
+  <si>
+    <t xml:space="preserve">张琦 主编</t>
+  </si>
+  <si>
+    <t xml:space="preserve">978-7-5080-7825-0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hxph.com.cn/allBooks/3899.jhtml</t>
+  </si>
+  <si>
     <t xml:space="preserve">运动疗法技术学</t>
   </si>
   <si>
@@ -14625,6 +14782,78 @@
   </si>
   <si>
     <t xml:space="preserve">https://lib.zy91.com/opac/book/38902</t>
+  </si>
+  <si>
+    <t xml:space="preserve">运动疗法与作业疗法</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">于兑生</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">恽晓平 编著</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">978-7-5080-7857-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hxph.com.cn/newBooks/9290.jhtml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">水中运动疗法手册</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">侯晓晖</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">王珅 主编</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">978-7-5080-8998-0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.hxph.com.cn/allBooks/6302.jhtml</t>
   </si>
   <si>
     <t xml:space="preserve">厦门大学出版社</t>
@@ -23216,7 +23445,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -25172,11 +25401,9 @@
       <c r="C48" s="4" t="s">
         <v>1296</v>
       </c>
-      <c r="D48" s="5" t="s">
-        <v>1091</v>
-      </c>
+      <c r="D48" s="2"/>
       <c r="E48" s="2" t="n">
-        <v>2011</v>
+        <v>2023</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>1297</v>
@@ -25191,19 +25418,19 @@
         <v>1298</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="M48" s="9" t="s">
         <v>229</v>
       </c>
       <c r="N48" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="O48" s="7" t="s">
         <v>1299</v>
       </c>
-      <c r="O48" s="7" t="s">
-        <v>1300</v>
-      </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="n">
         <v>48</v>
       </c>
@@ -25211,35 +25438,43 @@
         <v>1295</v>
       </c>
       <c r="C49" s="4" t="s">
+        <v>1300</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>1096</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F49" s="3" t="s">
         <v>1301</v>
       </c>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="F49" s="4" t="s">
+      <c r="G49" s="4" t="s">
         <v>1302</v>
       </c>
-      <c r="G49" s="3"/>
       <c r="H49" s="5" t="s">
-        <v>1070</v>
-      </c>
-      <c r="I49" s="3"/>
-      <c r="J49" s="2"/>
+        <v>1099</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>1303</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>1245</v>
+      </c>
       <c r="K49" s="2" t="s">
-        <v>1303</v>
+        <v>1304</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="M49" s="6" t="s">
-        <v>26</v>
+        <v>81</v>
+      </c>
+      <c r="M49" s="9" t="s">
+        <v>229</v>
       </c>
       <c r="N49" s="5" t="s">
         <v>318</v>
       </c>
       <c r="O49" s="7" t="s">
-        <v>1304</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25247,17 +25482,19 @@
         <v>49</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>1305</v>
+        <v>1295</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D50" s="2"/>
+        <v>1306</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>1091</v>
+      </c>
       <c r="E50" s="2" t="n">
-        <v>2016</v>
+        <v>2014</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>1306</v>
+        <v>1307</v>
       </c>
       <c r="G50" s="3"/>
       <c r="H50" s="5" t="s">
@@ -25265,7 +25502,9 @@
       </c>
       <c r="I50" s="3"/>
       <c r="J50" s="2"/>
-      <c r="K50" s="2"/>
+      <c r="K50" s="2" t="s">
+        <v>1308</v>
+      </c>
       <c r="L50" s="5" t="s">
         <v>25</v>
       </c>
@@ -25276,7 +25515,7 @@
         <v>318</v>
       </c>
       <c r="O50" s="7" t="s">
-        <v>1307</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25284,17 +25523,19 @@
         <v>50</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>1308</v>
+        <v>1295</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>1309</v>
-      </c>
-      <c r="D51" s="2"/>
+        <v>1310</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>1091</v>
+      </c>
       <c r="E51" s="2" t="n">
-        <v>2023</v>
+        <v>2011</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>1310</v>
+        <v>1311</v>
       </c>
       <c r="G51" s="3"/>
       <c r="H51" s="5" t="s">
@@ -25303,19 +25544,19 @@
       <c r="I51" s="3"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2" t="s">
-        <v>1311</v>
+        <v>1312</v>
       </c>
       <c r="L51" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="M51" s="8" t="s">
-        <v>38</v>
+        <v>25</v>
+      </c>
+      <c r="M51" s="9" t="s">
+        <v>229</v>
       </c>
       <c r="N51" s="5" t="s">
-        <v>318</v>
+        <v>1313</v>
       </c>
       <c r="O51" s="7" t="s">
-        <v>1312</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25323,17 +25564,17 @@
         <v>51</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>1313</v>
+        <v>1295</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>1314</v>
+        <v>1315</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>1315</v>
+        <v>1316</v>
       </c>
       <c r="G52" s="3"/>
       <c r="H52" s="5" t="s">
@@ -25342,16 +25583,16 @@
       <c r="I52" s="3"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2" t="s">
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="M52" s="9" t="s">
-        <v>229</v>
+      <c r="M52" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="N52" s="5" t="s">
-        <v>1317</v>
+        <v>318</v>
       </c>
       <c r="O52" s="7" t="s">
         <v>1318</v>
@@ -25362,17 +25603,19 @@
         <v>52</v>
       </c>
       <c r="B53" s="5" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C53" s="4" t="s">
         <v>1319</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="D53" s="5" t="s">
+        <v>1091</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F53" s="4" t="s">
         <v>1320</v>
-      </c>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="F53" s="4" t="s">
-        <v>1321</v>
       </c>
       <c r="G53" s="3"/>
       <c r="H53" s="5" t="s">
@@ -25381,60 +25624,58 @@
       <c r="I53" s="3"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="L53" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="M53" s="8" t="s">
-        <v>38</v>
+      <c r="M53" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="N53" s="5" t="s">
         <v>318</v>
       </c>
       <c r="O53" s="7" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>1319</v>
+        <v>1295</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="F54" s="3" t="s">
-        <v>1325</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>1326</v>
-      </c>
+        <v>2017</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>1324</v>
+      </c>
+      <c r="G54" s="3"/>
       <c r="H54" s="5" t="s">
-        <v>1099</v>
+        <v>1070</v>
       </c>
       <c r="I54" s="3"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="L54" s="5" t="s">
-        <v>1115</v>
-      </c>
-      <c r="M54" s="9" t="s">
-        <v>229</v>
+        <v>25</v>
+      </c>
+      <c r="M54" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="N54" s="5" t="s">
         <v>318</v>
       </c>
       <c r="O54" s="7" t="s">
-        <v>1328</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25442,17 +25683,17 @@
         <v>54</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>1329</v>
+        <v>1327</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>1330</v>
+        <v>25</v>
       </c>
       <c r="D55" s="2"/>
       <c r="E55" s="2" t="n">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>1331</v>
+        <v>1328</v>
       </c>
       <c r="G55" s="3"/>
       <c r="H55" s="5" t="s">
@@ -25460,11 +25701,9 @@
       </c>
       <c r="I55" s="3"/>
       <c r="J55" s="2"/>
-      <c r="K55" s="2" t="s">
-        <v>1332</v>
-      </c>
+      <c r="K55" s="2"/>
       <c r="L55" s="5" t="s">
-        <v>195</v>
+        <v>25</v>
       </c>
       <c r="M55" s="9" t="s">
         <v>229</v>
@@ -25473,7 +25712,7 @@
         <v>318</v>
       </c>
       <c r="O55" s="7" t="s">
-        <v>1333</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25481,17 +25720,17 @@
         <v>55</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>1334</v>
+        <v>1331</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="2" t="n">
-        <v>2019</v>
+        <v>2023</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>1335</v>
+        <v>1332</v>
       </c>
       <c r="G56" s="3"/>
       <c r="H56" s="5" t="s">
@@ -25500,19 +25739,19 @@
       <c r="I56" s="3"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2" t="s">
-        <v>1336</v>
+        <v>1333</v>
       </c>
       <c r="L56" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="M56" s="9" t="s">
-        <v>229</v>
+        <v>37</v>
+      </c>
+      <c r="M56" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="N56" s="5" t="s">
         <v>318</v>
       </c>
       <c r="O56" s="7" t="s">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25520,42 +25759,38 @@
         <v>56</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>1329</v>
+        <v>1335</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="F57" s="3" t="s">
-        <v>1339</v>
+        <v>2023</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>1337</v>
       </c>
       <c r="G57" s="3"/>
       <c r="H57" s="5" t="s">
-        <v>1099</v>
-      </c>
-      <c r="I57" s="3" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I57" s="3"/>
+      <c r="J57" s="2"/>
+      <c r="K57" s="2" t="s">
+        <v>1338</v>
+      </c>
+      <c r="L57" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="M57" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="N57" s="5" t="s">
+        <v>1339</v>
+      </c>
+      <c r="O57" s="7" t="s">
         <v>1340</v>
-      </c>
-      <c r="J57" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="K57" s="2" t="s">
-        <v>1341</v>
-      </c>
-      <c r="L57" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="M57" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="N57" s="5" t="s">
-        <v>318</v>
-      </c>
-      <c r="O57" s="7" t="s">
-        <v>1342</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25563,19 +25798,17 @@
         <v>57</v>
       </c>
       <c r="B58" s="5" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>1342</v>
+      </c>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F58" s="4" t="s">
         <v>1343</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>1344</v>
-      </c>
-      <c r="D58" s="5" t="s">
-        <v>1345</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>2020</v>
-      </c>
-      <c r="F58" s="4" t="s">
-        <v>1118</v>
       </c>
       <c r="G58" s="3"/>
       <c r="H58" s="5" t="s">
@@ -25584,10 +25817,10 @@
       <c r="I58" s="3"/>
       <c r="J58" s="2"/>
       <c r="K58" s="2" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="L58" s="5" t="s">
-        <v>1115</v>
+        <v>37</v>
       </c>
       <c r="M58" s="8" t="s">
         <v>38</v>
@@ -25596,48 +25829,48 @@
         <v>318</v>
       </c>
       <c r="O58" s="7" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
       <c r="C59" s="4" t="s">
+        <v>1346</v>
+      </c>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>1347</v>
+      </c>
+      <c r="G59" s="4" t="s">
         <v>1348</v>
       </c>
-      <c r="D59" s="5" t="s">
-        <v>1091</v>
-      </c>
-      <c r="E59" s="2" t="n">
-        <v>2019</v>
-      </c>
-      <c r="F59" s="4" t="s">
-        <v>1349</v>
-      </c>
-      <c r="G59" s="3"/>
       <c r="H59" s="5" t="s">
-        <v>1070</v>
+        <v>1099</v>
       </c>
       <c r="I59" s="3"/>
       <c r="J59" s="2"/>
       <c r="K59" s="2" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="L59" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="M59" s="8" t="s">
-        <v>38</v>
+        <v>1115</v>
+      </c>
+      <c r="M59" s="9" t="s">
+        <v>229</v>
       </c>
       <c r="N59" s="5" t="s">
         <v>318</v>
       </c>
       <c r="O59" s="7" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25645,14 +25878,14 @@
         <v>59</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>1343</v>
+        <v>1351</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>1352</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2" t="n">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>1353</v>
@@ -25667,7 +25900,7 @@
         <v>1354</v>
       </c>
       <c r="L60" s="5" t="s">
-        <v>37</v>
+        <v>195</v>
       </c>
       <c r="M60" s="9" t="s">
         <v>229</v>
@@ -25684,14 +25917,14 @@
         <v>60</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>1343</v>
+        <v>1351</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>1356</v>
       </c>
       <c r="D61" s="2"/>
       <c r="E61" s="2" t="n">
-        <v>2022</v>
+        <v>2019</v>
       </c>
       <c r="F61" s="4" t="s">
         <v>1357</v>
@@ -25706,7 +25939,7 @@
         <v>1358</v>
       </c>
       <c r="L61" s="5" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="M61" s="9" t="s">
         <v>229</v>
@@ -25723,29 +25956,33 @@
         <v>61</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>1343</v>
+        <v>1351</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>1360</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="2" t="n">
-        <v>2010</v>
-      </c>
-      <c r="F62" s="4" t="s">
+        <v>2022</v>
+      </c>
+      <c r="F62" s="3" t="s">
         <v>1361</v>
       </c>
       <c r="G62" s="3"/>
       <c r="H62" s="5" t="s">
-        <v>1070</v>
-      </c>
-      <c r="I62" s="3"/>
-      <c r="J62" s="2"/>
+        <v>1099</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>1362</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="K62" s="2" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>1115</v>
+        <v>228</v>
       </c>
       <c r="M62" s="6" t="s">
         <v>26</v>
@@ -25754,7 +25991,7 @@
         <v>318</v>
       </c>
       <c r="O62" s="7" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -25762,17 +25999,19 @@
         <v>62</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>1343</v>
+        <v>1365</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>1364</v>
-      </c>
-      <c r="D63" s="2"/>
+        <v>1366</v>
+      </c>
+      <c r="D63" s="5" t="s">
+        <v>1367</v>
+      </c>
       <c r="E63" s="2" t="n">
-        <v>2010</v>
+        <v>2020</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>1365</v>
+        <v>1118</v>
       </c>
       <c r="G63" s="3"/>
       <c r="H63" s="5" t="s">
@@ -25781,56 +26020,54 @@
       <c r="I63" s="3"/>
       <c r="J63" s="2"/>
       <c r="K63" s="2" t="s">
-        <v>1366</v>
+        <v>1368</v>
       </c>
       <c r="L63" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="M63" s="6" t="s">
-        <v>26</v>
+        <v>1115</v>
+      </c>
+      <c r="M63" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="N63" s="5" t="s">
         <v>318</v>
       </c>
       <c r="O63" s="7" t="s">
-        <v>1367</v>
+        <v>1369</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="n">
         <v>63</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>1368</v>
+        <v>1365</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>1369</v>
-      </c>
-      <c r="D64" s="2"/>
+        <v>1370</v>
+      </c>
+      <c r="D64" s="5" t="s">
+        <v>1091</v>
+      </c>
       <c r="E64" s="2" t="n">
-        <v>2021</v>
-      </c>
-      <c r="F64" s="3" t="s">
-        <v>1370</v>
-      </c>
-      <c r="G64" s="4" t="s">
+        <v>2019</v>
+      </c>
+      <c r="F64" s="4" t="s">
         <v>1371</v>
       </c>
+      <c r="G64" s="3"/>
       <c r="H64" s="5" t="s">
-        <v>1099</v>
-      </c>
-      <c r="I64" s="3" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I64" s="3"/>
+      <c r="J64" s="2"/>
+      <c r="K64" s="2" t="s">
         <v>1372</v>
       </c>
-      <c r="J64" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="K64" s="2"/>
       <c r="L64" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="M64" s="9" t="s">
-        <v>229</v>
+        <v>25</v>
+      </c>
+      <c r="M64" s="8" t="s">
+        <v>38</v>
       </c>
       <c r="N64" s="5" t="s">
         <v>318</v>
@@ -25839,8 +26076,207 @@
         <v>1373</v>
       </c>
     </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="5" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>1374</v>
+      </c>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>1375</v>
+      </c>
+      <c r="G65" s="3"/>
+      <c r="H65" s="5" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I65" s="3"/>
+      <c r="J65" s="2"/>
+      <c r="K65" s="2" t="s">
+        <v>1376</v>
+      </c>
+      <c r="L65" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M65" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="N65" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="O65" s="7" t="s">
+        <v>1377</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="5" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>1378</v>
+      </c>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>1379</v>
+      </c>
+      <c r="G66" s="3"/>
+      <c r="H66" s="5" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I66" s="3"/>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2" t="s">
+        <v>1380</v>
+      </c>
+      <c r="L66" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M66" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="N66" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="O66" s="7" t="s">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="5" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>1382</v>
+      </c>
+      <c r="D67" s="2"/>
+      <c r="E67" s="2" t="n">
+        <v>2010</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>1383</v>
+      </c>
+      <c r="G67" s="3"/>
+      <c r="H67" s="5" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I67" s="3"/>
+      <c r="J67" s="2"/>
+      <c r="K67" s="2" t="s">
+        <v>1384</v>
+      </c>
+      <c r="L67" s="5" t="s">
+        <v>1115</v>
+      </c>
+      <c r="M67" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N67" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="O67" s="7" t="s">
+        <v>1385</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="5" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>1386</v>
+      </c>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2" t="n">
+        <v>2010</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>1387</v>
+      </c>
+      <c r="G68" s="3"/>
+      <c r="H68" s="5" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I68" s="3"/>
+      <c r="J68" s="2"/>
+      <c r="K68" s="2" t="s">
+        <v>1388</v>
+      </c>
+      <c r="L68" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="M68" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="N68" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="O68" s="7" t="s">
+        <v>1389</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>1390</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>1391</v>
+      </c>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>1392</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>1393</v>
+      </c>
+      <c r="H69" s="5" t="s">
+        <v>1099</v>
+      </c>
+      <c r="I69" s="3" t="s">
+        <v>1394</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="K69" s="2"/>
+      <c r="L69" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="M69" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="N69" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="O69" s="7" t="s">
+        <v>1395</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O64"/>
+  <autoFilter ref="A1:O69"/>
   <hyperlinks>
     <hyperlink ref="O2" r:id="rId1" display="https://wyutsg.wuyiu.edu.cn/mspace/searchDetailLocal/m82e8999ce9a845eaf40f14ad495ee365"/>
     <hyperlink ref="O3" r:id="rId2" display="https://lib.zy91.com/opac/book/40536"/>
@@ -25888,23 +26324,28 @@
     <hyperlink ref="O45" r:id="rId44" display="https://lib.zy91.com/opac/book/39185"/>
     <hyperlink ref="O46" r:id="rId45" display="https://lib.zy91.com/opac/book/34321"/>
     <hyperlink ref="O47" r:id="rId46" display="https://lib.zy91.com/opac/book/30341"/>
-    <hyperlink ref="O48" r:id="rId47" display="https://opac.bsu.edu.cn/mspace/searchDetailLocal/m15df5c7cebf4b9ba4cf1d3c6ba0d1245"/>
-    <hyperlink ref="O49" r:id="rId48" display="https://lib.zy91.com/opac/book/38902"/>
-    <hyperlink ref="O50" r:id="rId49" display="https://book.douban.com/subject/30268830/"/>
-    <hyperlink ref="O51" r:id="rId50" display="https://tsgopac.sdxd.edu.cn:17453/mspace/searchDetailLocal/m89518776e5a397999f21248ee809301c"/>
-    <hyperlink ref="O52" r:id="rId51" display="https://opac.bsu.edu.cn/mspace/searchDetailLocal/me04b86c68f279542aff18721ef2f3fb5"/>
-    <hyperlink ref="O53" r:id="rId52" display="http://www.csmu.edu.cn:8081/ILASOPAC/NTRdrBookRetr.do?SearchType=text&amp;SearchKey=%25E4%25B8%25BB%25E7%25BC%2596&amp;leftAuthorType=author&amp;leftAuthorKey=%E5%AE%B9%E5%8F%AF%EF%BC%8C%E6%9D%8E%E5%B0%8F%E5%85%AD%E4%B8%BB%E7%BC%96%EF%BC%9B"/>
-    <hyperlink ref="O54" r:id="rId53" display="https://yjsjy.symc.edu.cn/info/3621/11652.htm"/>
-    <hyperlink ref="O55" r:id="rId54" display="https://lib.zy91.com/opac/book/36545"/>
-    <hyperlink ref="O56" r:id="rId55" display="https://opac.bsu.edu.cn/mspace/searchDetailLocal/ma33a9b4255d9836dc228d490ac2cdf1a"/>
-    <hyperlink ref="O57" r:id="rId56" display="https://lib.zy91.com/opac/book/39013"/>
-    <hyperlink ref="O58" r:id="rId57" display="https://lib.tjh.com.cn/mspace/searchDetailLocal/m87da0ed576ae53980be71e06c5b86d12"/>
-    <hyperlink ref="O59" r:id="rId58" display="https://opac.bsu.edu.cn/mspace/searchDetailLocal/m6a96577e8640f51ee4b1496ce15d7d84"/>
-    <hyperlink ref="O60" r:id="rId59" display="https://www.megbook.com.hk/mall/detail.jsp?proID=3912725"/>
-    <hyperlink ref="O61" r:id="rId60" display="https://lib.zy91.com/opac/book/36180"/>
-    <hyperlink ref="O62" r:id="rId61" display="https://lib.zy91.com/opac/book/25785"/>
-    <hyperlink ref="O63" r:id="rId62" display="https://lib.zy91.com/opac/book/25783"/>
-    <hyperlink ref="O64" r:id="rId63" display="https://book.douban.com/subject/35676782/"/>
+    <hyperlink ref="O48" r:id="rId47" display="https://www.hxph.com.cn/newBooks/9475.jhtml"/>
+    <hyperlink ref="O49" r:id="rId48" display="https://www.hxph.com.cn/newBooks/8974.jhtml"/>
+    <hyperlink ref="O50" r:id="rId49" display="https://www.hxph.com.cn/allBooks/3899.jhtml"/>
+    <hyperlink ref="O51" r:id="rId50" display="https://opac.bsu.edu.cn/mspace/searchDetailLocal/m15df5c7cebf4b9ba4cf1d3c6ba0d1245"/>
+    <hyperlink ref="O52" r:id="rId51" display="https://lib.zy91.com/opac/book/38902"/>
+    <hyperlink ref="O53" r:id="rId52" display="https://www.hxph.com.cn/newBooks/9290.jhtml"/>
+    <hyperlink ref="O54" r:id="rId53" display="https://www.hxph.com.cn/allBooks/6302.jhtml"/>
+    <hyperlink ref="O55" r:id="rId54" display="https://book.douban.com/subject/30268830/"/>
+    <hyperlink ref="O56" r:id="rId55" display="https://tsgopac.sdxd.edu.cn:17453/mspace/searchDetailLocal/m89518776e5a397999f21248ee809301c"/>
+    <hyperlink ref="O57" r:id="rId56" display="https://opac.bsu.edu.cn/mspace/searchDetailLocal/me04b86c68f279542aff18721ef2f3fb5"/>
+    <hyperlink ref="O58" r:id="rId57" display="http://www.csmu.edu.cn:8081/ILASOPAC/NTRdrBookRetr.do?SearchType=text&amp;SearchKey=%25E4%25B8%25BB%25E7%25BC%2596&amp;leftAuthorType=author&amp;leftAuthorKey=%E5%AE%B9%E5%8F%AF%EF%BC%8C%E6%9D%8E%E5%B0%8F%E5%85%AD%E4%B8%BB%E7%BC%96%EF%BC%9B"/>
+    <hyperlink ref="O59" r:id="rId58" display="https://yjsjy.symc.edu.cn/info/3621/11652.htm"/>
+    <hyperlink ref="O60" r:id="rId59" display="https://lib.zy91.com/opac/book/36545"/>
+    <hyperlink ref="O61" r:id="rId60" display="https://opac.bsu.edu.cn/mspace/searchDetailLocal/ma33a9b4255d9836dc228d490ac2cdf1a"/>
+    <hyperlink ref="O62" r:id="rId61" display="https://lib.zy91.com/opac/book/39013"/>
+    <hyperlink ref="O63" r:id="rId62" display="https://lib.tjh.com.cn/mspace/searchDetailLocal/m87da0ed576ae53980be71e06c5b86d12"/>
+    <hyperlink ref="O64" r:id="rId63" display="https://opac.bsu.edu.cn/mspace/searchDetailLocal/m6a96577e8640f51ee4b1496ce15d7d84"/>
+    <hyperlink ref="O65" r:id="rId64" display="https://www.megbook.com.hk/mall/detail.jsp?proID=3912725"/>
+    <hyperlink ref="O66" r:id="rId65" display="https://lib.zy91.com/opac/book/36180"/>
+    <hyperlink ref="O67" r:id="rId66" display="https://lib.zy91.com/opac/book/25785"/>
+    <hyperlink ref="O68" r:id="rId67" display="https://lib.zy91.com/opac/book/25783"/>
+    <hyperlink ref="O69" r:id="rId68" display="https://book.douban.com/subject/35676782/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -25913,7 +26354,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <drawing r:id="rId64"/>
+  <drawing r:id="rId69"/>
 </worksheet>
 </file>
 
@@ -25931,35 +26372,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>1374</v>
+        <v>1396</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>1375</v>
+        <v>1397</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>1376</v>
+        <v>1398</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>1377</v>
+        <v>1399</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>1378</v>
+        <v>1400</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>1379</v>
+        <v>1401</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>1380</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26081,7 +26522,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>1381</v>
+        <v>1403</v>
       </c>
       <c r="B21" s="11" t="n">
         <f aca="false">SUM(B8:B20)</f>
@@ -26090,15 +26531,15 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>1382</v>
+        <v>1404</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
-        <v>1379</v>
+        <v>1401</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>1380</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26130,7 +26571,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>1381</v>
+        <v>1403</v>
       </c>
       <c r="B28" s="11" t="n">
         <f aca="false">SUM(B25:B27)</f>
@@ -26139,15 +26580,15 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>1383</v>
+        <v>1405</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>1379</v>
+        <v>1401</v>
       </c>
       <c r="B31" s="13" t="s">
-        <v>1380</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26155,7 +26596,7 @@
         <v>1067</v>
       </c>
       <c r="B32" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A32)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A32)</f>
         <v>1</v>
       </c>
     </row>
@@ -26164,7 +26605,7 @@
         <v>1073</v>
       </c>
       <c r="B33" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A33)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A33)</f>
         <v>2</v>
       </c>
     </row>
@@ -26173,7 +26614,7 @@
         <v>1082</v>
       </c>
       <c r="B34" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A34)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A34)</f>
         <v>3</v>
       </c>
     </row>
@@ -26182,7 +26623,7 @@
         <v>1094</v>
       </c>
       <c r="B35" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A35)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A35)</f>
         <v>5</v>
       </c>
     </row>
@@ -26191,7 +26632,7 @@
         <v>1121</v>
       </c>
       <c r="B36" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A36)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A36)</f>
         <v>15</v>
       </c>
     </row>
@@ -26200,7 +26641,7 @@
         <v>1195</v>
       </c>
       <c r="B37" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A37)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A37)</f>
         <v>2</v>
       </c>
     </row>
@@ -26209,7 +26650,7 @@
         <v>1204</v>
       </c>
       <c r="B38" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A38)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A38)</f>
         <v>6</v>
       </c>
     </row>
@@ -26218,7 +26659,7 @@
         <v>1228</v>
       </c>
       <c r="B39" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A39)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A39)</f>
         <v>4</v>
       </c>
     </row>
@@ -26227,7 +26668,7 @@
         <v>1252</v>
       </c>
       <c r="B40" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A40)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A40)</f>
         <v>8</v>
       </c>
     </row>
@@ -26236,93 +26677,93 @@
         <v>1295</v>
       </c>
       <c r="B41" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A41)</f>
-        <v>2</v>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A41)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="15" t="s">
-        <v>1305</v>
+        <v>1327</v>
       </c>
       <c r="B42" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A42)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A42)</f>
         <v>1</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="15" t="s">
-        <v>1308</v>
+        <v>1330</v>
       </c>
       <c r="B43" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A43)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A43)</f>
         <v>1</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="15" t="s">
-        <v>1313</v>
+        <v>1335</v>
       </c>
       <c r="B44" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A44)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A44)</f>
         <v>1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="15" t="s">
-        <v>1319</v>
+        <v>1341</v>
       </c>
       <c r="B45" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A45)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A45)</f>
         <v>2</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="15" t="s">
-        <v>1329</v>
+        <v>1351</v>
       </c>
       <c r="B46" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A46)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A46)</f>
         <v>3</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="15" t="s">
-        <v>1343</v>
+        <v>1365</v>
       </c>
       <c r="B47" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A47)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A47)</f>
         <v>6</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="15" t="s">
-        <v>1368</v>
+        <v>1390</v>
       </c>
       <c r="B48" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$B$2:$B$64,A48)</f>
+        <f aca="false">COUNTIF(中文出版社!$B$2:$B$69,A48)</f>
         <v>1</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>1381</v>
+        <v>1403</v>
       </c>
       <c r="B49" s="11" t="n">
         <f aca="false">SUM(B32:B48)</f>
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>1384</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="13" t="s">
-        <v>1379</v>
+        <v>1401</v>
       </c>
       <c r="B52" s="13" t="s">
-        <v>1380</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26330,8 +26771,8 @@
         <v>1070</v>
       </c>
       <c r="B53" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$H$2:$H$64,A53)</f>
-        <v>34</v>
+        <f aca="false">COUNTIF(中文出版社!$H$2:$H$69,A53)</f>
+        <v>38</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26339,30 +26780,30 @@
         <v>1099</v>
       </c>
       <c r="B54" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$H$2:$H$64,A54)</f>
-        <v>27</v>
+        <f aca="false">COUNTIF(中文出版社!$H$2:$H$69,A54)</f>
+        <v>28</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>1381</v>
+        <v>1403</v>
       </c>
       <c r="B55" s="11" t="n">
         <f aca="false">SUM(B53:B54)</f>
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>1385</v>
+        <v>1407</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="13" t="s">
-        <v>1379</v>
+        <v>1401</v>
       </c>
       <c r="B58" s="13" t="s">
-        <v>1380</v>
+        <v>1402</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26370,7 +26811,7 @@
         <v>38</v>
       </c>
       <c r="B59" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$M$2:$M$64,A59)</f>
+        <f aca="false">COUNTIF(中文出版社!$M$2:$M$69,A59)</f>
         <v>26</v>
       </c>
     </row>
@@ -26379,8 +26820,8 @@
         <v>229</v>
       </c>
       <c r="B60" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$M$2:$M$64,A60)</f>
-        <v>27</v>
+        <f aca="false">COUNTIF(中文出版社!$M$2:$M$69,A60)</f>
+        <v>30</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26388,17 +26829,17 @@
         <v>26</v>
       </c>
       <c r="B61" s="14" t="n">
-        <f aca="false">COUNTIF(中文出版社!$M$2:$M$64,A61)</f>
-        <v>10</v>
+        <f aca="false">COUNTIF(中文出版社!$M$2:$M$69,A61)</f>
+        <v>12</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="11" t="s">
-        <v>1381</v>
+        <v>1403</v>
       </c>
       <c r="B62" s="11" t="n">
         <f aca="false">SUM(B59:B61)</f>
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>